<commit_message>
feat: implement OOP architecture and Filler class: - Created 'Filler' class module to handle range populations - Added private state management for pversion and pDefaultValue - Implemented error handling with centralized 'Handler' sub - Updated 'main' to use Object-oriented approach instead of direct cell manipulation - Standardized use of Range and Cells objects
</commit_message>
<xml_diff>
--- a/.vba/learning.xlsx
+++ b/.vba/learning.xlsx
@@ -5,26 +5,57 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario Pc\Desktop\learning\VBA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario Pc\Desktop\learning\.vba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFADDDFA-3E3F-4C89-A99F-43923BF2B24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E96089D-EA71-4DD8-BEBC-9BA47D9050DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="720" yWindow="735" windowWidth="19530" windowHeight="9540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -43,7 +74,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -58,6 +89,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -442,8 +479,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A2:D5"/>
+  <dimension ref="A2:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
@@ -456,6 +496,12 @@
       </c>
       <c r="C5" s="1" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C7" t="e" cm="1">
+        <f t="array" ref="C7">square(2)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>